<commit_message>
fix: clean up duplicate BADGE_ICON_PATHS block
</commit_message>
<xml_diff>
--- a/media/Media List.xlsx
+++ b/media/Media List.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10703"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/DornellesDa/commonwealth-explorer/media/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{948FC962-2ACE-8340-8482-8D05EDD4DF47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{254B1488-972C-4741-A601-5419353D220B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5180" yWindow="4280" windowWidth="26840" windowHeight="15680" xr2:uid="{E56E0FED-61F8-5540-8A37-9A20088EE8C5}"/>
+    <workbookView xWindow="420" yWindow="1620" windowWidth="26840" windowHeight="15680" xr2:uid="{E56E0FED-61F8-5540-8A37-9A20088EE8C5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,14 +39,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="20">
   <si>
     <t>Country</t>
   </si>
   <si>
-    <t>Youtube Link</t>
-  </si>
-  <si>
     <t>Pakistan</t>
   </si>
   <si>
@@ -59,40 +56,49 @@
     <t>© Colourful Heritage. Used with permission.</t>
   </si>
   <si>
-    <t xml:space="preserve">https://www.colourfulheritage.com/portfolio/bashirmaan2013/ </t>
-  </si>
-  <si>
-    <t>https://www.colourfulheritage.com/portfolio/shaheenunis/ </t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.colourfulheritage.com/portfolio/mr-ashaque-ali/ </t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.colourfulheritage.com/portfolio/mrs-zubaidah-azad/ </t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.colourfulheritage.com/portfolio/mohammadsarwar/ </t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.colourfulheritage.com/portfolio/mrs-perveen-sarwar/ </t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.colourfulheritage.com/portfolio/mr-darbara-singh-bhullar/ </t>
-  </si>
-  <si>
     <t>India</t>
   </si>
   <si>
-    <t xml:space="preserve">https://www.colourfulheritage.com/portfolio/mrs_daljit_kaur_dilber/ </t>
-  </si>
-  <si>
-    <t>https://www.colourfulheritage.com/portfolio/sawarnjit-matharu/</t>
-  </si>
-  <si>
-    <t>https://www.colourfulheritage.com/portfolio/herstory-sawarnjit-matharu/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.colourfulheritage.com/portfolio/prof_brajraman_sinha/ </t>
+    <t>Title</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Link</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=teUtBOeaVto</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=8F8t4lrouss</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=_mD8EX5ZAJI</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=9dZt-cH-dvU</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=hEc_is0QfKw</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=yvm1-GJX7zM</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=uVuoobNV55A</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=yhqLG_mO8MM</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=x0szVB4KNPU</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=9wcUi7wL8OI</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=_3iy4IaDXzI</t>
   </si>
 </sst>
 </file>
@@ -483,169 +489,172 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F4D20EB-093E-5E40-9C2E-056F114D9EB9}">
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="60.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.83203125" customWidth="1"/>
+    <col min="4" max="4" width="60.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+      <c r="D2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2" t="s">
+      <c r="E2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>1</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>1</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>1</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>1</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E7" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>1</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E8" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="D9" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E9" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" t="s">
+      <c r="D10" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E10" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>2</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C5" t="s">
+      <c r="D11" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E11" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>2</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C6" t="s">
+      <c r="D12" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E12" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>2</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C7" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>2</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="C8" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>13</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C9" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>13</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C10" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>13</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C11" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="C12" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
-        <v>13</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C13" t="s">
-        <v>5</v>
+      <c r="D13" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E13" t="s">
+        <v>4</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1" xr:uid="{FDEE42B9-41FD-3E4F-A03B-D222F81B46BB}"/>
-    <hyperlink ref="B3" r:id="rId2" xr:uid="{F2236D28-9BEB-0F43-BE81-CBF49E049418}"/>
-    <hyperlink ref="B4" r:id="rId3" display="https://www.colourfulheritage.com/portfolio/shaheenunis/" xr:uid="{353C84A1-7A95-ED4F-8E8E-E57C7DB43D93}"/>
-    <hyperlink ref="B5" r:id="rId4" xr:uid="{59810E1C-AC0F-2C4C-8F8B-1FD9D76D2275}"/>
-    <hyperlink ref="B6" r:id="rId5" xr:uid="{D1C3973C-0BCB-E64B-A39F-D00A48DB9D94}"/>
-    <hyperlink ref="B7" r:id="rId6" xr:uid="{EB262BD9-4841-3445-A4ED-73EB6EFC899A}"/>
-    <hyperlink ref="B8" r:id="rId7" xr:uid="{C2F53D04-8E47-734E-BFBC-7C3AEE9F83C5}"/>
-    <hyperlink ref="B9" r:id="rId8" xr:uid="{D9CD25BB-1637-5445-A8C3-C188AABB7912}"/>
-    <hyperlink ref="B10" r:id="rId9" xr:uid="{A1A871EF-2DD8-264B-AAF6-D1A7884797E0}"/>
-    <hyperlink ref="B11" r:id="rId10" xr:uid="{687D0B70-0085-B64D-8321-2DCA793108DA}"/>
-    <hyperlink ref="B12" r:id="rId11" xr:uid="{F45383A3-8068-7148-8884-7151E1232E8E}"/>
-    <hyperlink ref="B13" r:id="rId12" xr:uid="{311B5909-30E4-C541-B0C2-0A4DE0A7722C}"/>
+    <hyperlink ref="D2" r:id="rId1" xr:uid="{FDEE42B9-41FD-3E4F-A03B-D222F81B46BB}"/>
+    <hyperlink ref="D3" r:id="rId2" xr:uid="{F2236D28-9BEB-0F43-BE81-CBF49E049418}"/>
+    <hyperlink ref="D4" r:id="rId3" xr:uid="{353C84A1-7A95-ED4F-8E8E-E57C7DB43D93}"/>
+    <hyperlink ref="D5" r:id="rId4" xr:uid="{59810E1C-AC0F-2C4C-8F8B-1FD9D76D2275}"/>
+    <hyperlink ref="D6" r:id="rId5" xr:uid="{D1C3973C-0BCB-E64B-A39F-D00A48DB9D94}"/>
+    <hyperlink ref="D7" r:id="rId6" xr:uid="{EB262BD9-4841-3445-A4ED-73EB6EFC899A}"/>
+    <hyperlink ref="D8" r:id="rId7" xr:uid="{C2F53D04-8E47-734E-BFBC-7C3AEE9F83C5}"/>
+    <hyperlink ref="D12" r:id="rId8" xr:uid="{F45383A3-8068-7148-8884-7151E1232E8E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Fixes for player and modalities 2026
</commit_message>
<xml_diff>
--- a/media/Media List.xlsx
+++ b/media/Media List.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/DornellesDa/commonwealth-explorer/media/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{254B1488-972C-4741-A601-5419353D220B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{DE7D564C-11D0-F348-A7CD-10A7D354C545}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="420" yWindow="1620" windowWidth="26840" windowHeight="15680" xr2:uid="{E56E0FED-61F8-5540-8A37-9A20088EE8C5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="35">
   <si>
     <t>Country</t>
   </si>
@@ -65,9 +65,6 @@
     <t>Description</t>
   </si>
   <si>
-    <t xml:space="preserve"> Link</t>
-  </si>
-  <si>
     <t>https://www.youtube.com/watch?v=teUtBOeaVto</t>
   </si>
   <si>
@@ -99,6 +96,54 @@
   </si>
   <si>
     <t>https://www.youtube.com/watch?v=_3iy4IaDXzI</t>
+  </si>
+  <si>
+    <t>Youtube</t>
+  </si>
+  <si>
+    <t>CDN</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=H4oM8_eAzKI</t>
+  </si>
+  <si>
+    <t>https://videos.familysearch.fun/Bashir%20Maan%2C%20interviewed%20in%202011%20-%20Colourful%20Heritage%20(480p%2C%20h264%2C%20youtube).mp4</t>
+  </si>
+  <si>
+    <t>https://videos.familysearch.fun/Shaheen%20Unis%20-%20Colourful%20Heritage%20(480p%2C%20h264%2C%20youtube).mp4</t>
+  </si>
+  <si>
+    <t>https://videos.familysearch.fun/Mr%20Ashaque%20Ali%20-%20A%20Story%20of%20Family%2C%20Sacrifices%20and%20Hard%20Work%20-%20Colourful%20Heritage%20(1080p%2C%20h264%2C%20youtube).mp4</t>
+  </si>
+  <si>
+    <t>https://videos.familysearch.fun/Bashir%20Maan%2C%20interviewed%20in%202013%20-%20Colourful%20Heritage%20(720p%2C%20h264%2C%20youtube).mp4</t>
+  </si>
+  <si>
+    <t>https://videos.familysearch.fun/Mrs%20Zubaidah%20Azad%20-%20First%20South%20Asian%20Dux%20in%20Scotland%20-%20Colourful%20Heritage%20(1080p%2C%20h264%2C%20youtube)_1.mp4</t>
+  </si>
+  <si>
+    <t>https://videos.familysearch.fun/Mohammad%20Sarwar%20-%20Colourful%20Heritage%20(480p%2C%20h264%2C%20youtube).mp4</t>
+  </si>
+  <si>
+    <t>https://videos.familysearch.fun/Mrs%20Perveen%20Sarwar%20-%20Life%20in%20Early%20Lossiemouth%20-%20Colourful%20Heritage%20(1080p%2C%20h264%2C%20youtube).mp4</t>
+  </si>
+  <si>
+    <t>https://videos.familysearch.fun/Mr%20Darbara%20Singh%20Bhullar%20Part%201%20-%20Life%2C%20before%2C%20during%20and%20after%20partition%20-%20Colourful%20Heritage%20(1080p%2C%20h264%2C%20youtube).mp4</t>
+  </si>
+  <si>
+    <t>https://videos.familysearch.fun/Mrs%20Daljit%20Kaur%20Dilber%20Part%201%20-%20Journey%20to%20Glasgow%20and%20the%20sacrifices%20made%20-%20Colourful%20Heritage%20(1080p%2C%20h264%2C%20youtube).mp4</t>
+  </si>
+  <si>
+    <t>https://videos.familysearch.fun/Herstory%20-%20Sawarnjit%20Matharu%20-%20Colourful%20Heritage%20(1080p%20h264%20youtube).mp4</t>
+  </si>
+  <si>
+    <t>https://videos.familysearch.fun/Mrs%20Sawarnjit%20Matharu%20-%20It%20was%20all%20just%20very%20new%2C%20very%20different%20-%20Colourful%20Heritage%20(1080p%2C%20h264%2C%20youtube)_1.mp4</t>
+  </si>
+  <si>
+    <t>https://videos.familysearch.fun/Prof%20Brajraman%20Prasad%20Sinha%20Part%201%20Migration%20to%20the%20UK%20and%20academic%20career%20-%20Colourful%20Heritage%20(1080p%2C%20h264%2C%20youtube).mp4</t>
+  </si>
+  <si>
+    <t>https://videos.familysearch.fun/Dr%20Mohammad%20Kausar%20-%20Colourful%20Heritage%20(480p%2C%20h264%2C%20youtube).mp4</t>
   </si>
 </sst>
 </file>
@@ -489,14 +534,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F4D20EB-093E-5E40-9C2E-056F114D9EB9}">
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="14.83203125" customWidth="1"/>
     <col min="4" max="4" width="60.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="60.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -507,141 +553,194 @@
         <v>7</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="E1" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>1</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="E2" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>1</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E3" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="F3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>1</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E4" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+        <v>9</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>1</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E5" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="F5" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>1</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="E6" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+        <v>11</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="F6" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>1</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E7" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+        <v>12</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>1</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E8" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+        <v>13</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F8" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>5</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E9" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+        <v>14</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F9" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>5</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E10" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+        <v>15</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F10" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>5</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E11" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+        <v>16</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="F11" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>5</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="E12" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+        <v>17</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F12" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>5</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E13" t="s">
+        <v>18</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="F13" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>1</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F14" t="s">
         <v>4</v>
       </c>
     </row>
@@ -655,6 +754,22 @@
     <hyperlink ref="D7" r:id="rId6" xr:uid="{EB262BD9-4841-3445-A4ED-73EB6EFC899A}"/>
     <hyperlink ref="D8" r:id="rId7" xr:uid="{C2F53D04-8E47-734E-BFBC-7C3AEE9F83C5}"/>
     <hyperlink ref="D12" r:id="rId8" xr:uid="{F45383A3-8068-7148-8884-7151E1232E8E}"/>
+    <hyperlink ref="E2" r:id="rId9" xr:uid="{6F7BC87B-8C28-2F4B-8D0B-D968EA64EDCA}"/>
+    <hyperlink ref="E4" r:id="rId10" xr:uid="{54BFE6BA-0479-A346-84E0-52F17346E6DC}"/>
+    <hyperlink ref="E5" r:id="rId11" xr:uid="{7BA24605-8D42-1D48-A92F-794B15E11972}"/>
+    <hyperlink ref="E3" r:id="rId12" xr:uid="{25AFA94F-F05E-4647-9885-E8BE1847477B}"/>
+    <hyperlink ref="E7" r:id="rId13" xr:uid="{7B9F0D13-8D6F-9D4B-8731-735893B74FB1}"/>
+    <hyperlink ref="E8" r:id="rId14" xr:uid="{A330CE4A-7245-DD49-866C-BE33457C609F}"/>
+    <hyperlink ref="E10" r:id="rId15" xr:uid="{64632ACB-11AF-3443-824C-513FD951E748}"/>
+    <hyperlink ref="E11" r:id="rId16" xr:uid="{CAFF955B-70B7-FD49-953E-CF997BB501AE}"/>
+    <hyperlink ref="E12" r:id="rId17" xr:uid="{A02DFBBA-29FA-044C-AEBF-A841C4143E0A}"/>
+    <hyperlink ref="E13" r:id="rId18" xr:uid="{5ABAC1A0-7966-0D4F-BFAB-0C3F9FDB6A9C}"/>
+    <hyperlink ref="E14" r:id="rId19" xr:uid="{6F4C8390-19B2-F54B-8252-52AC5E73BBB8}"/>
+    <hyperlink ref="D9" r:id="rId20" xr:uid="{05FE1A34-02D5-4291-9900-24DEB1D81356}"/>
+    <hyperlink ref="D10" r:id="rId21" xr:uid="{FD9A65AD-543B-47FF-8F6C-E108E79D2AA6}"/>
+    <hyperlink ref="D11" r:id="rId22" xr:uid="{33AF785D-44D4-49A0-8174-E3B33579189C}"/>
+    <hyperlink ref="D13" r:id="rId23" xr:uid="{B3CB1AD5-770E-45F9-A3FF-DDA40078BC83}"/>
+    <hyperlink ref="D14" r:id="rId24" xr:uid="{33BD44DA-1536-4F44-90A6-7E474AE23022}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>